<commit_message>
changing auto increment...and update directorate_id to be required in supervisors
</commit_message>
<xml_diff>
--- a/Reports/supervisors_names_2026.xlsx
+++ b/Reports/supervisors_names_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IMC_1\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IMC_1\Documents\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F276AFD9-C175-4F73-9DA3-ADD1AE0737FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4EA984-41DD-4B87-A776-7705E1E4A11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E8F31610-7129-4F8B-8402-3462BE0584F5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>SuperVisor_Name</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>user</t>
+  </si>
+  <si>
+    <t>directorate_id</t>
   </si>
 </sst>
 </file>
@@ -521,10 +524,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4FD4A8-4223-492E-A0E5-D9D551470ED8}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -534,269 +537,371 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D11">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
       <c r="C14" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>16</v>
       </c>
       <c r="C15" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D15">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>17</v>
       </c>
       <c r="C16" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>18</v>
       </c>
       <c r="C17" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>19</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>20</v>
       </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D19">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
       <c r="C20" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D20">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>22</v>
       </c>
       <c r="C21" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D21">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>23</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D22">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>24</v>
       </c>
       <c r="C23" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D23">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>25</v>
       </c>
       <c r="C24" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D24">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>26</v>
       </c>
       <c r="C25" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D25">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>27</v>
       </c>
       <c r="C26" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D26">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>28</v>
       </c>
       <c r="C27" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D27">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>29</v>
       </c>
       <c r="C28" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D28">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>30</v>
       </c>
       <c r="C29" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D29">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D30">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D31">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>33</v>
       </c>
       <c r="C32" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D32">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D33">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>35</v>
       </c>
       <c r="C34" t="s">
         <v>36</v>
+      </c>
+      <c r="D34">
+        <v>1411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update the schools list
</commit_message>
<xml_diff>
--- a/Reports/supervisors_names_2026.xlsx
+++ b/Reports/supervisors_names_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IMC_1\Documents\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4EA984-41DD-4B87-A776-7705E1E4A11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D14679B-C742-47BE-BCE5-16468BE6FF0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E8F31610-7129-4F8B-8402-3462BE0584F5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{E8F31610-7129-4F8B-8402-3462BE0584F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="39">
   <si>
     <t>SuperVisor_Name</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>directorate_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuperVisor_id </t>
   </si>
 </sst>
 </file>
@@ -524,387 +527,493 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE4FD4A8-4223-492E-A0E5-D9D551470ED8}">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="30.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1411</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="D2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2">
+        <v>979962172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1411</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3">
+        <v>984551242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1411</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="D4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4">
+        <v>986202810</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1411</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5">
+        <v>946770856</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1411</v>
+      </c>
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6">
+        <v>925061046</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1411</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7">
+        <v>979955267</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1411</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="D8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8">
+        <v>900129834</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1411</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9">
+        <v>850917824</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1411</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10">
+        <v>907323976</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1411</v>
+      </c>
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11">
+        <v>999824154</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1411</v>
+      </c>
+      <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12">
+        <v>921716064</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1411</v>
+      </c>
+      <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="D13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13">
+        <v>901043265</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1411</v>
+      </c>
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14">
+        <v>991195934</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1411</v>
+      </c>
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="C15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15">
+        <v>904131711</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1411</v>
+      </c>
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16">
+        <v>914096532</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1411</v>
+      </c>
+      <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="C17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="D17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17">
+        <v>978348415</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1411</v>
+      </c>
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18">
+        <v>938845674</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1411</v>
+      </c>
+      <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="D19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19">
+        <v>905653242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1411</v>
+      </c>
+      <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="C20" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20">
+        <v>904117991</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1411</v>
+      </c>
+      <c r="B21" t="s">
         <v>22</v>
       </c>
-      <c r="C21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21">
+        <v>913206124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1411</v>
+      </c>
+      <c r="B22" t="s">
         <v>23</v>
       </c>
-      <c r="C22" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22">
+        <v>901237537</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1411</v>
+      </c>
+      <c r="B23" t="s">
         <v>24</v>
       </c>
-      <c r="C23" t="s">
-        <v>36</v>
-      </c>
-      <c r="D23">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23">
+        <v>851149054</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>1411</v>
+      </c>
+      <c r="B24" t="s">
         <v>25</v>
       </c>
-      <c r="C24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24">
+        <v>943281733</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>1411</v>
+      </c>
+      <c r="B25" t="s">
         <v>26</v>
       </c>
-      <c r="C25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25">
+        <v>946042892</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>1411</v>
+      </c>
+      <c r="B26" t="s">
         <v>27</v>
       </c>
-      <c r="C26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="D26" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26">
+        <v>904199080</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>1411</v>
+      </c>
+      <c r="B27" t="s">
         <v>28</v>
       </c>
-      <c r="C27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D27">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27">
+        <v>995395233</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>1411</v>
+      </c>
+      <c r="B28" t="s">
         <v>29</v>
       </c>
-      <c r="C28" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28">
+        <v>961337839</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>1411</v>
+      </c>
+      <c r="B29" t="s">
         <v>30</v>
       </c>
-      <c r="C29" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="D29" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29">
+        <v>904072170</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>1411</v>
+      </c>
+      <c r="B30" t="s">
         <v>31</v>
       </c>
-      <c r="C30" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="D30" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30">
+        <v>904995800</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>1411</v>
+      </c>
+      <c r="B31" t="s">
         <v>32</v>
       </c>
-      <c r="C31" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="D31" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31">
+        <v>904439197</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>1411</v>
+      </c>
+      <c r="B32" t="s">
         <v>33</v>
       </c>
-      <c r="C32" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="D32" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32">
+        <v>906183322</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>1411</v>
+      </c>
+      <c r="B33" t="s">
         <v>34</v>
       </c>
-      <c r="C33" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33">
-        <v>1411</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="D33" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33">
+        <v>994328565</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>1411</v>
+      </c>
+      <c r="B34" t="s">
         <v>35</v>
       </c>
-      <c r="C34" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34">
-        <v>1411</v>
+      <c r="D34" t="s">
+        <v>36</v>
+      </c>
+      <c r="E34">
+        <v>850644378</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>